<commit_message>
Add company financial API endpoints
</commit_message>
<xml_diff>
--- a/reports/peer_comparison.xlsx
+++ b/reports/peer_comparison.xlsx
@@ -604,22 +604,22 @@
         </is>
       </c>
       <c r="G2" s="1" t="n">
-        <v>9.51</v>
+        <v>9.50809964894472</v>
       </c>
       <c r="H2" s="1" t="n">
-        <v>13</v>
+        <v>13.13003143989059</v>
       </c>
       <c r="I2" s="1" t="n">
-        <v>15.75</v>
+        <v>15.75038535195478</v>
       </c>
       <c r="J2" s="1" t="n">
-        <v>0.0014</v>
+        <v>0.001389602503619973</v>
       </c>
       <c r="K2" s="1" t="n">
-        <v>117.9072</v>
+        <v>117.9072164948454</v>
       </c>
       <c r="L2" s="1" t="n">
-        <v>1.2303</v>
+        <v>1.230295566502463</v>
       </c>
       <c r="M2" s="1" t="n">
         <v>4936</v>
@@ -686,22 +686,22 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>7.26</v>
+        <v>7.263066074788551</v>
       </c>
       <c r="H3" t="n">
-        <v>14</v>
+        <v>13.59538554282896</v>
       </c>
       <c r="I3" t="n">
-        <v>37.46</v>
+        <v>37.45613415294755</v>
       </c>
       <c r="J3" t="n">
-        <v>1.2631</v>
+        <v>1.263124425916767</v>
       </c>
       <c r="K3" t="n">
-        <v>6.5302</v>
+        <v>6.530242339274985</v>
       </c>
       <c r="L3" t="n">
-        <v>1.1851</v>
+        <v>1.185123443593192</v>
       </c>
       <c r="M3" t="n">
         <v>45133</v>
@@ -769,22 +769,22 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>8.82</v>
+        <v>8.822387437265419</v>
       </c>
       <c r="H4" t="n">
-        <v>18</v>
+        <v>17.89787025985418</v>
       </c>
       <c r="I4" t="n">
-        <v>18.54</v>
+        <v>18.53754343556428</v>
       </c>
       <c r="J4" t="n">
-        <v>1.6414</v>
+        <v>1.641441305333132</v>
       </c>
       <c r="K4" t="n">
-        <v>3.7647</v>
+        <v>3.764690170940171</v>
       </c>
       <c r="L4" t="n">
-        <v>0.5925</v>
+        <v>0.5925222177725139</v>
       </c>
       <c r="M4" t="n">
         <v>-11245</v>
@@ -851,22 +851,22 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>17.18</v>
+        <v>17.17851571205706</v>
       </c>
       <c r="H5" t="n">
-        <v>20</v>
+        <v>19.53420993982616</v>
       </c>
       <c r="I5" t="n">
-        <v>26.61</v>
+        <v>26.61418410330778</v>
       </c>
       <c r="J5" t="n">
-        <v>0.066</v>
+        <v>0.06601754022512257</v>
       </c>
       <c r="K5" t="n">
-        <v>174.4167</v>
+        <v>174.4166666666667</v>
       </c>
       <c r="L5" t="n">
-        <v>1.1405</v>
+        <v>1.140453436356242</v>
       </c>
       <c r="M5" t="n">
         <v>6486</v>
@@ -933,22 +933,22 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>24.2</v>
+        <v>24.19569424286405</v>
       </c>
       <c r="H6" t="n">
-        <v>26</v>
+        <v>26.17924528301887</v>
       </c>
       <c r="I6" t="n">
-        <v>22.17</v>
+        <v>22.17234691050152</v>
       </c>
       <c r="J6" t="n">
-        <v>0.0232</v>
+        <v>0.02321972845663619</v>
       </c>
       <c r="K6" t="n">
-        <v>114.7059</v>
+        <v>114.7058823529412</v>
       </c>
       <c r="L6" t="n">
-        <v>0.7154</v>
+        <v>0.7153796236210254</v>
       </c>
       <c r="M6" t="n">
         <v>890</v>
@@ -1016,22 +1016,22 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>9.9</v>
+        <v>9.902352536452407</v>
       </c>
       <c r="H7" t="n">
-        <v>5235</v>
+        <v>86.14676228532112</v>
       </c>
       <c r="I7" t="n">
-        <v>21.14</v>
+        <v>21.14243742584327</v>
       </c>
       <c r="J7" t="n">
-        <v>0.0342</v>
+        <v>0.03423922255494661</v>
       </c>
       <c r="K7" t="n">
-        <v>47.2685</v>
+        <v>47.26850507982584</v>
       </c>
       <c r="L7" t="n">
-        <v>1.4449</v>
+        <v>1.444920276832486</v>
       </c>
       <c r="M7" t="n">
         <v>3095</v>
@@ -1098,22 +1098,22 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>4.54</v>
+        <v>4.544641716694342</v>
       </c>
       <c r="H8" t="n">
-        <v>14</v>
+        <v>14.05032571209605</v>
       </c>
       <c r="I8" t="n">
-        <v>26.22</v>
+        <v>26.22346698113208</v>
       </c>
       <c r="J8" t="n">
-        <v>3.8334</v>
+        <v>3.833431603773585</v>
       </c>
       <c r="K8" t="n">
-        <v>2.9077</v>
+        <v>2.907676348547718</v>
       </c>
       <c r="L8" t="n">
-        <v>0.9315</v>
+        <v>0.9314915286502951</v>
       </c>
       <c r="M8" t="n">
         <v>-2254</v>
@@ -1168,7 +1168,7 @@
         <v>9.51</v>
       </c>
       <c r="H9" t="n">
-        <v>18</v>
+        <v>17.9</v>
       </c>
       <c r="I9" t="n">
         <v>22.17</v>
@@ -1423,22 +1423,22 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>15.94</v>
+        <v>15.93948250956673</v>
       </c>
       <c r="H3" t="n">
-        <v>4102</v>
+        <v>37.4889127294537</v>
       </c>
       <c r="I3" t="n">
-        <v>15.76</v>
+        <v>15.7618637908999</v>
       </c>
       <c r="J3" t="n">
-        <v>12.1437</v>
+        <v>12.14371872728943</v>
       </c>
       <c r="K3" t="n">
-        <v>1.8967</v>
+        <v>1.896747724261721</v>
       </c>
       <c r="L3" t="n">
-        <v>0.07149999999999999</v>
+        <v>0.07153782236255685</v>
       </c>
       <c r="M3" t="n">
         <v>-7559</v>
@@ -1505,22 +1505,22 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>13.94</v>
+        <v>13.93516047014541</v>
       </c>
       <c r="H4" t="n">
-        <v>-7745</v>
+        <v>41.75390656810141</v>
       </c>
       <c r="I4" t="n">
-        <v>16.72</v>
+        <v>16.71605179468811</v>
       </c>
       <c r="J4" t="n">
-        <v>14.8674</v>
+        <v>14.86741992554242</v>
       </c>
       <c r="K4" t="n">
-        <v>1.6107</v>
+        <v>1.610661174334986</v>
       </c>
       <c r="L4" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.0719985042520674</v>
       </c>
       <c r="M4" t="n">
         <v>13296</v>
@@ -1587,16 +1587,16 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>8.4</v>
+        <v>8.395910695456838</v>
       </c>
       <c r="I5" t="n">
-        <v>61.31999999999999</v>
+        <v>61.32056519118731</v>
       </c>
       <c r="J5" t="n">
-        <v>3.6843</v>
+        <v>3.684256345007701</v>
       </c>
       <c r="L5" t="n">
-        <v>1.507</v>
+        <v>1.50702629506294</v>
       </c>
       <c r="M5" t="n">
         <v>-29445</v>
@@ -1648,7 +1648,7 @@
         <v>13.94</v>
       </c>
       <c r="H6" t="n">
-        <v>-1821.5</v>
+        <v>39.62</v>
       </c>
       <c r="I6" t="n">
         <v>16.72</v>
@@ -1864,22 +1864,22 @@
         </is>
       </c>
       <c r="G2" s="1" t="n">
-        <v>-2.14</v>
+        <v>-2.142504941724738</v>
       </c>
       <c r="H2" s="1" t="n">
-        <v>10</v>
+        <v>9.708034611709159</v>
       </c>
       <c r="I2" s="1" t="n">
-        <v>-5.33</v>
+        <v>-5.334926929972293</v>
       </c>
       <c r="J2" s="1" t="n">
-        <v>0.9462</v>
+        <v>0.9461835171402184</v>
       </c>
       <c r="K2" s="1" t="n">
-        <v>2.1634</v>
+        <v>2.16342567927544</v>
       </c>
       <c r="L2" s="1" t="n">
-        <v>0.8509</v>
+        <v>0.8509498277091255</v>
       </c>
       <c r="M2" s="1" t="n">
         <v>6048</v>
@@ -1946,22 +1946,22 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>5.13</v>
+        <v>5.127252779904689</v>
       </c>
       <c r="H3" t="n">
-        <v>16</v>
+        <v>16.08916265728032</v>
       </c>
       <c r="I3" t="n">
-        <v>11.55</v>
+        <v>11.5528718021347</v>
       </c>
       <c r="J3" t="n">
-        <v>1.1328</v>
+        <v>1.132807168883338</v>
       </c>
       <c r="K3" t="n">
-        <v>3.6591</v>
+        <v>3.659099321406539</v>
       </c>
       <c r="L3" t="n">
-        <v>0.7679</v>
+        <v>0.7679137157851319</v>
       </c>
       <c r="M3" t="n">
         <v>-2389</v>
@@ -2028,22 +2028,22 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>11.8</v>
+        <v>11.80243873376494</v>
       </c>
       <c r="H4" t="n">
-        <v>20</v>
+        <v>20.26055526869762</v>
       </c>
       <c r="I4" t="n">
-        <v>13.41</v>
+        <v>13.4105063633902</v>
       </c>
       <c r="J4" t="n">
-        <v>0.3717</v>
+        <v>0.3716941962270963</v>
       </c>
       <c r="K4" t="n">
-        <v>8.0046</v>
+        <v>8.004636785162287</v>
       </c>
       <c r="L4" t="n">
-        <v>0.64</v>
+        <v>0.6400172860847018</v>
       </c>
       <c r="M4" t="n">
         <v>-2336</v>
@@ -2110,22 +2110,22 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>4.7</v>
+        <v>4.702216130615571</v>
       </c>
       <c r="H5" t="n">
-        <v>23872</v>
+        <v>88.94620349876368</v>
       </c>
       <c r="I5" t="n">
-        <v>9.57</v>
+        <v>9.567011474761177</v>
       </c>
       <c r="J5" t="n">
-        <v>0.5309</v>
+        <v>0.5309290976579428</v>
       </c>
       <c r="K5" t="n">
-        <v>126.4654</v>
+        <v>126.4654377880184</v>
       </c>
       <c r="L5" t="n">
-        <v>0.9360000000000001</v>
+        <v>0.9360228499109322</v>
       </c>
       <c r="M5" t="n">
         <v>9789</v>
@@ -2177,10 +2177,10 @@
         <v>665</v>
       </c>
       <c r="G6" t="n">
-        <v>4.92</v>
+        <v>4.91</v>
       </c>
       <c r="H6" t="n">
-        <v>18</v>
+        <v>18.17</v>
       </c>
       <c r="I6" t="n">
         <v>10.56</v>
@@ -2395,22 +2395,22 @@
         </is>
       </c>
       <c r="G2" s="1" t="n">
-        <v>26.29</v>
+        <v>26.28792839991269</v>
       </c>
       <c r="H2" s="1" t="n">
-        <v>19987</v>
+        <v>29.28581823473769</v>
       </c>
       <c r="I2" s="1" t="n">
-        <v>18.84</v>
+        <v>18.8419213518306</v>
       </c>
       <c r="J2" s="1" t="n">
-        <v>3.8248</v>
+        <v>3.824788776468134</v>
       </c>
       <c r="K2" s="1" t="n">
-        <v>2689.1667</v>
+        <v>2689.166666666667</v>
       </c>
       <c r="L2" s="1" t="n">
-        <v>0.1463</v>
+        <v>0.1463025160881669</v>
       </c>
       <c r="M2" s="1" t="n">
         <v>-79931</v>
@@ -2477,22 +2477,22 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>17.85</v>
+        <v>17.84689244899024</v>
       </c>
       <c r="H3" t="n">
-        <v>4548</v>
+        <v>28.10102802275218</v>
       </c>
       <c r="I3" t="n">
-        <v>17.46</v>
+        <v>17.45521359669269</v>
       </c>
       <c r="J3" t="n">
-        <v>6.8634</v>
+        <v>6.863420609401317</v>
       </c>
       <c r="K3" t="n">
-        <v>21.2118</v>
+        <v>21.21176470588235</v>
       </c>
       <c r="L3" t="n">
-        <v>0.1223</v>
+        <v>0.1223019286981607</v>
       </c>
       <c r="M3" t="n">
         <v>-38538</v>
@@ -2560,22 +2560,22 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>20.33</v>
+        <v>20.33362647026492</v>
       </c>
       <c r="H4" t="n">
-        <v>29</v>
+        <v>28.9188743541827</v>
       </c>
       <c r="I4" t="n">
-        <v>15.12</v>
+        <v>15.11635033812082</v>
       </c>
       <c r="J4" t="n">
-        <v>3.994</v>
+        <v>3.994034363699512</v>
       </c>
       <c r="K4" t="n">
-        <v>0.6767</v>
+        <v>0.6766743648960739</v>
       </c>
       <c r="L4" t="n">
-        <v>0.1466</v>
+        <v>0.1465685998082702</v>
       </c>
       <c r="M4" t="n">
         <v>-31359</v>
@@ -2630,7 +2630,7 @@
         <v>20.33</v>
       </c>
       <c r="H5" t="n">
-        <v>4548</v>
+        <v>28.92</v>
       </c>
       <c r="I5" t="n">
         <v>17.46</v>
@@ -2846,22 +2846,22 @@
         </is>
       </c>
       <c r="G2" s="1" t="n">
-        <v>16.61</v>
+        <v>16.61173581491534</v>
       </c>
       <c r="H2" s="1" t="n">
-        <v>14659</v>
+        <v>76.31672482874498</v>
       </c>
       <c r="I2" s="1" t="n">
-        <v>20.07</v>
+        <v>20.07497364207896</v>
       </c>
       <c r="J2" s="1" t="n">
-        <v>0.029</v>
+        <v>0.02897418876176344</v>
       </c>
       <c r="K2" s="1" t="n">
-        <v>57.847</v>
+        <v>57.8470012239902</v>
       </c>
       <c r="L2" s="1" t="n">
-        <v>0.7886</v>
+        <v>0.7885945801322478</v>
       </c>
       <c r="M2" s="1" t="n">
         <v>10145</v>
@@ -2929,22 +2929,22 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>29.28</v>
+        <v>29.28202523071713</v>
       </c>
       <c r="H3" t="n">
-        <v>37</v>
+        <v>37.0177518132814</v>
       </c>
       <c r="I3" t="n">
-        <v>27.85</v>
+        <v>27.85107439569436</v>
       </c>
       <c r="J3" t="n">
-        <v>0.0041</v>
+        <v>0.004066731984914169</v>
       </c>
       <c r="K3" t="n">
         <v>362.9625</v>
       </c>
       <c r="L3" t="n">
-        <v>0.7723</v>
+        <v>0.7723477995509732</v>
       </c>
       <c r="M3" t="n">
         <v>18742</v>
@@ -3011,22 +3011,22 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>12.73</v>
+        <v>12.72586319995229</v>
       </c>
       <c r="H4" t="n">
-        <v>19</v>
+        <v>18.88603971614288</v>
       </c>
       <c r="I4" t="n">
-        <v>54.15</v>
+        <v>54.14869322506978</v>
       </c>
       <c r="J4" t="n">
-        <v>0.524</v>
+        <v>0.5239786856127886</v>
       </c>
       <c r="K4" t="n">
-        <v>20.5976</v>
+        <v>20.59756097560976</v>
       </c>
       <c r="L4" t="n">
-        <v>1.8484</v>
+        <v>1.848434744268078</v>
       </c>
       <c r="M4" t="n">
         <v>3050</v>
@@ -3093,22 +3093,22 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>14.6</v>
+        <v>14.60012899064818</v>
       </c>
       <c r="H5" t="n">
-        <v>19</v>
+        <v>19.34859722670106</v>
       </c>
       <c r="I5" t="n">
-        <v>18.36</v>
+        <v>18.35596999797284</v>
       </c>
       <c r="J5" t="n">
-        <v>0.1384</v>
+        <v>0.1383539428339753</v>
       </c>
       <c r="K5" t="n">
-        <v>23.2419</v>
+        <v>23.24193548387097</v>
       </c>
       <c r="L5" t="n">
-        <v>0.8206</v>
+        <v>0.8205874569992061</v>
       </c>
       <c r="M5" t="n">
         <v>1042</v>
@@ -3175,22 +3175,22 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>16.12</v>
+        <v>16.12281708616873</v>
       </c>
       <c r="H6" t="n">
-        <v>24</v>
+        <v>23.82963023694351</v>
       </c>
       <c r="I6" t="n">
-        <v>117.75</v>
+        <v>117.7544910179641</v>
       </c>
       <c r="J6" t="n">
-        <v>0.1033</v>
+        <v>0.1032934131736527</v>
       </c>
       <c r="K6" t="n">
-        <v>41.1862</v>
+        <v>41.18620689655172</v>
       </c>
       <c r="L6" t="n">
-        <v>2.3182</v>
+        <v>2.318160220469448</v>
       </c>
       <c r="M6" t="n">
         <v>2938</v>
@@ -3257,22 +3257,22 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>-3.98</v>
+        <v>-3.979852440408627</v>
       </c>
       <c r="H7" t="n">
-        <v>21</v>
+        <v>20.97758229284904</v>
       </c>
       <c r="I7" t="n">
-        <v>-4.45</v>
+        <v>-4.45308779171297</v>
       </c>
       <c r="J7" t="n">
-        <v>0.2558</v>
+        <v>0.2557548817272583</v>
       </c>
       <c r="K7" t="n">
-        <v>2.4129</v>
+        <v>2.412903225806452</v>
       </c>
       <c r="L7" t="n">
-        <v>0.7664</v>
+        <v>0.7664201826881253</v>
       </c>
       <c r="M7" t="n">
         <v>-1365</v>
@@ -3336,22 +3336,22 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>7.99</v>
+        <v>7.990266999868473</v>
       </c>
       <c r="H8" t="n">
-        <v>15</v>
+        <v>15.02038668946468</v>
       </c>
       <c r="I8" t="n">
-        <v>7.57</v>
+        <v>7.566793298872766</v>
       </c>
       <c r="J8" t="n">
-        <v>0.2165</v>
+        <v>0.21654107242947</v>
       </c>
       <c r="K8" t="n">
-        <v>25.3218</v>
+        <v>25.32183908045977</v>
       </c>
       <c r="L8" t="n">
-        <v>0.5454</v>
+        <v>0.5454284586965099</v>
       </c>
       <c r="M8" t="n">
         <v>26</v>
@@ -3406,7 +3406,7 @@
         <v>14.6</v>
       </c>
       <c r="H9" t="n">
-        <v>21</v>
+        <v>20.98</v>
       </c>
       <c r="I9" t="n">
         <v>20.07</v>
@@ -3621,22 +3621,22 @@
         </is>
       </c>
       <c r="G2" s="1" t="n">
-        <v>19.14</v>
+        <v>19.13671215020777</v>
       </c>
       <c r="H2" s="1" t="n">
-        <v>27</v>
+        <v>26.69068839692312</v>
       </c>
       <c r="I2" s="1" t="n">
-        <v>50.94</v>
+        <v>50.94431367348518</v>
       </c>
       <c r="J2" s="1" t="n">
-        <v>0.0886</v>
+        <v>0.0886406082507266</v>
       </c>
       <c r="K2" s="1" t="n">
-        <v>87.0951</v>
+        <v>87.09511568123393</v>
       </c>
       <c r="L2" s="1" t="n">
-        <v>1.6559</v>
+        <v>1.655940662120545</v>
       </c>
       <c r="M2" s="1" t="n">
         <v>50429</v>
@@ -3703,22 +3703,22 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>17.08</v>
+        <v>17.08075746730006</v>
       </c>
       <c r="H3" t="n">
-        <v>24</v>
+        <v>23.70339038198738</v>
       </c>
       <c r="I3" t="n">
-        <v>29.79</v>
+        <v>29.78800671841663</v>
       </c>
       <c r="J3" t="n">
-        <v>0.0949</v>
+        <v>0.09486358890553362</v>
       </c>
       <c r="K3" t="n">
-        <v>87.5234</v>
+        <v>87.52340425531915</v>
       </c>
       <c r="L3" t="n">
-        <v>1.1298</v>
+        <v>1.129760329363329</v>
       </c>
       <c r="M3" t="n">
         <v>20117</v>
@@ -3782,22 +3782,22 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>14.29</v>
+        <v>14.29312274253273</v>
       </c>
       <c r="H4" t="n">
-        <v>22</v>
+        <v>22.01559415173819</v>
       </c>
       <c r="I4" t="n">
-        <v>23.01</v>
+        <v>23.01393141233172</v>
       </c>
       <c r="J4" t="n">
-        <v>0.0844</v>
+        <v>0.08435023365512796</v>
       </c>
       <c r="K4" t="n">
-        <v>46.4611</v>
+        <v>46.46112115732369</v>
       </c>
       <c r="L4" t="n">
-        <v>1.1102</v>
+        <v>1.110165040502596</v>
       </c>
       <c r="M4" t="n">
         <v>15840</v>
@@ -3864,22 +3864,22 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>4.61</v>
+        <v>4.60996999769213</v>
       </c>
       <c r="H5" t="n">
-        <v>9</v>
+        <v>8.666051234710363</v>
       </c>
       <c r="I5" t="n">
-        <v>8.99</v>
+        <v>8.987963553189097</v>
       </c>
       <c r="J5" t="n">
-        <v>0.0951</v>
+        <v>0.09512917619708275</v>
       </c>
       <c r="K5" t="n">
-        <v>13.8597</v>
+        <v>13.85969387755102</v>
       </c>
       <c r="L5" t="n">
-        <v>1.205</v>
+        <v>1.205033720364319</v>
       </c>
       <c r="M5" t="n">
         <v>5058</v>
@@ -3946,22 +3946,22 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>12.91</v>
+        <v>12.90931103415266</v>
       </c>
       <c r="H6" t="n">
-        <v>18</v>
+        <v>17.98293774812062</v>
       </c>
       <c r="I6" t="n">
-        <v>22.9</v>
+        <v>22.9043860525527</v>
       </c>
       <c r="J6" t="n">
-        <v>0.1035</v>
+        <v>0.1034568888000799</v>
       </c>
       <c r="K6" t="n">
-        <v>31.9324</v>
+        <v>31.93243243243243</v>
       </c>
       <c r="L6" t="n">
-        <v>1.2895</v>
+        <v>1.289464130119082</v>
       </c>
       <c r="M6" t="n">
         <v>1752</v>
@@ -4016,7 +4016,7 @@
         <v>14.29</v>
       </c>
       <c r="H7" t="n">
-        <v>22</v>
+        <v>22.02</v>
       </c>
       <c r="I7" t="n">
         <v>23.01</v>
@@ -4028,7 +4028,7 @@
         <v>46.46</v>
       </c>
       <c r="L7" t="n">
-        <v>1.2</v>
+        <v>1.21</v>
       </c>
       <c r="M7" t="n">
         <v>15840</v>
@@ -4231,13 +4231,13 @@
         </is>
       </c>
       <c r="G2" s="1" t="n">
-        <v>4.84</v>
+        <v>4.836600998148862</v>
       </c>
       <c r="H2" s="1" t="n">
-        <v>4</v>
+        <v>3.87474201090824</v>
       </c>
       <c r="I2" s="1" t="n">
-        <v>49.45</v>
+        <v>49.44710986501021</v>
       </c>
       <c r="J2" s="1" t="n">
         <v>0</v>
@@ -4246,7 +4246,7 @@
         <v>371.9375</v>
       </c>
       <c r="L2" s="1" t="n">
-        <v>0.1591</v>
+        <v>0.1591344094587576</v>
       </c>
       <c r="M2" s="1" t="n">
         <v>853</v>
@@ -4313,22 +4313,22 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>1.55</v>
+        <v>1.551013972921306</v>
       </c>
       <c r="H3" t="n">
-        <v>531</v>
+        <v>99.47675449833469</v>
       </c>
       <c r="I3" t="n">
-        <v>10.73</v>
+        <v>10.73230601390972</v>
       </c>
       <c r="J3" t="n">
-        <v>0.0648</v>
+        <v>0.06477567162143734</v>
       </c>
       <c r="K3" t="n">
-        <v>192.2895</v>
+        <v>192.2895238095238</v>
       </c>
       <c r="L3" t="n">
-        <v>0.3353</v>
+        <v>0.3352704278677314</v>
       </c>
       <c r="M3" t="n">
         <v>-2893</v>
@@ -4395,22 +4395,22 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>1.43</v>
+        <v>1.434978937479165</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>0.1863805800527321</v>
       </c>
       <c r="I4" t="n">
-        <v>12.7</v>
+        <v>12.70458814059566</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>240.3333</v>
+        <v>240.3333333333333</v>
       </c>
       <c r="L4" t="n">
-        <v>0.3314</v>
+        <v>0.3313791900054984</v>
       </c>
       <c r="M4" t="n">
         <v>-2099</v>
@@ -4477,22 +4477,22 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.942341125272681</v>
       </c>
       <c r="H5" t="n">
-        <v>-1829</v>
+        <v>102.0253136523193</v>
       </c>
       <c r="I5" t="n">
-        <v>7.73</v>
+        <v>7.732848705134029</v>
       </c>
       <c r="J5" t="n">
-        <v>0.109</v>
+        <v>0.1090413448432531</v>
       </c>
       <c r="K5" t="n">
-        <v>31.0215</v>
+        <v>31.02154882154882</v>
       </c>
       <c r="L5" t="n">
-        <v>0.302</v>
+        <v>0.3020290902037117</v>
       </c>
       <c r="M5" t="n">
         <v>105</v>
@@ -4547,7 +4547,7 @@
         <v>1.49</v>
       </c>
       <c r="H6" t="n">
-        <v>2</v>
+        <v>51.68</v>
       </c>
       <c r="I6" t="n">
         <v>11.72</v>
@@ -4763,22 +4763,22 @@
         </is>
       </c>
       <c r="G2" s="1" t="n">
-        <v>8.790000000000001</v>
+        <v>8.789365557299389</v>
       </c>
       <c r="H2" s="1" t="n">
-        <v>18</v>
+        <v>18.07459281612296</v>
       </c>
       <c r="I2" s="1" t="n">
-        <v>9.960000000000001</v>
+        <v>9.958650553699458</v>
       </c>
       <c r="J2" s="1" t="n">
-        <v>0.5785</v>
+        <v>0.5784524141094746</v>
       </c>
       <c r="K2" s="1" t="n">
-        <v>7.7289</v>
+        <v>7.728912535686478</v>
       </c>
       <c r="L2" s="1" t="n">
-        <v>0.5123</v>
+        <v>0.5122600635424216</v>
       </c>
       <c r="M2" s="1" t="n">
         <v>45207</v>
@@ -4845,22 +4845,22 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>9.66</v>
+        <v>9.655290194725701</v>
       </c>
       <c r="H3" t="n">
-        <v>17</v>
+        <v>17.38851801500179</v>
       </c>
       <c r="I3" t="n">
-        <v>16.94</v>
+        <v>16.94039813688551</v>
       </c>
       <c r="J3" t="n">
-        <v>0.4544</v>
+        <v>0.4544486308481918</v>
       </c>
       <c r="K3" t="n">
-        <v>11.3613</v>
+        <v>11.361290955464</v>
       </c>
       <c r="L3" t="n">
-        <v>0.8332000000000001</v>
+        <v>0.8332173339682772</v>
       </c>
       <c r="M3" t="n">
         <v>42060</v>
@@ -4927,22 +4927,22 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>5.99</v>
+        <v>5.994201967046283</v>
       </c>
       <c r="H4" t="n">
-        <v>10</v>
+        <v>9.837909494446341</v>
       </c>
       <c r="I4" t="n">
-        <v>35.51000000000001</v>
+        <v>35.51133734382231</v>
       </c>
       <c r="J4" t="n">
-        <v>0.7219</v>
+        <v>0.7218747934157467</v>
       </c>
       <c r="K4" t="n">
-        <v>11.3555</v>
+        <v>11.35550735116896</v>
       </c>
       <c r="L4" t="n">
-        <v>2.2137</v>
+        <v>2.213651947949293</v>
       </c>
       <c r="M4" t="n">
         <v>25415</v>
@@ -5010,22 +5010,22 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>5.56</v>
+        <v>5.559462717942377</v>
       </c>
       <c r="H5" t="n">
-        <v>10</v>
+        <v>9.743776019125345</v>
       </c>
       <c r="I5" t="n">
-        <v>23.53</v>
+        <v>23.53162465856491</v>
       </c>
       <c r="J5" t="n">
-        <v>0.7231</v>
+        <v>0.7230954600718581</v>
       </c>
       <c r="K5" t="n">
-        <v>10.2823</v>
+        <v>10.28232457809923</v>
       </c>
       <c r="L5" t="n">
-        <v>1.6084</v>
+        <v>1.608409660170339</v>
       </c>
       <c r="M5" t="n">
         <v>39635</v>
@@ -5092,22 +5092,22 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>7.430000000000001</v>
+        <v>7.433122166511544</v>
       </c>
       <c r="H6" t="n">
-        <v>11</v>
+        <v>10.74398775032275</v>
       </c>
       <c r="I6" t="n">
-        <v>12.86</v>
+        <v>12.86154006000234</v>
       </c>
       <c r="J6" t="n">
-        <v>0.283</v>
+        <v>0.2830499889606088</v>
       </c>
       <c r="K6" t="n">
-        <v>23.6245</v>
+        <v>23.62447844228095</v>
       </c>
       <c r="L6" t="n">
-        <v>1.0681</v>
+        <v>1.068088347296268</v>
       </c>
       <c r="M6" t="n">
         <v>4360</v>
@@ -5162,7 +5162,7 @@
         <v>7.43</v>
       </c>
       <c r="H7" t="n">
-        <v>11</v>
+        <v>10.74</v>
       </c>
       <c r="I7" t="n">
         <v>16.94</v>
@@ -5377,22 +5377,22 @@
         </is>
       </c>
       <c r="G2" s="1" t="n">
-        <v>19.82</v>
+        <v>19.81565870053818</v>
       </c>
       <c r="H2" s="1" t="n">
-        <v>28</v>
+        <v>26.84289749881436</v>
       </c>
       <c r="I2" s="1" t="n">
-        <v>15.09</v>
+        <v>15.09416181067115</v>
       </c>
       <c r="J2" s="1" t="n">
-        <v>0.0514</v>
+        <v>0.05142381453500244</v>
       </c>
       <c r="K2" s="1" t="n">
-        <v>58.3319</v>
+        <v>58.33193277310924</v>
       </c>
       <c r="L2" s="1" t="n">
-        <v>0.5685</v>
+        <v>0.5684929901064378</v>
       </c>
       <c r="M2" s="1" t="n">
         <v>11372</v>
@@ -5460,22 +5460,22 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>16.12</v>
+        <v>16.11701714906495</v>
       </c>
       <c r="H3" t="n">
-        <v>6291</v>
+        <v>75.59168153953597</v>
       </c>
       <c r="I3" t="n">
-        <v>15.55</v>
+        <v>15.55455702838313</v>
       </c>
       <c r="J3" t="n">
-        <v>0.0209</v>
+        <v>0.02093162585186849</v>
       </c>
       <c r="K3" t="n">
-        <v>35.3388</v>
+        <v>35.33876811594203</v>
       </c>
       <c r="L3" t="n">
-        <v>0.7922</v>
+        <v>0.7922417237881536</v>
       </c>
       <c r="M3" t="n">
         <v>1152</v>
@@ -5542,22 +5542,22 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>19.91</v>
+        <v>19.9136053693192</v>
       </c>
       <c r="H4" t="n">
-        <v>28</v>
+        <v>28.32101674342223</v>
       </c>
       <c r="I4" t="n">
-        <v>19.74</v>
+        <v>19.74233736816026</v>
       </c>
       <c r="J4" t="n">
-        <v>0.0709</v>
+        <v>0.07085722375592836</v>
       </c>
       <c r="K4" t="n">
-        <v>51.7076</v>
+        <v>51.70760233918129</v>
       </c>
       <c r="L4" t="n">
-        <v>0.7223000000000001</v>
+        <v>0.7223053120165034</v>
       </c>
       <c r="M4" t="n">
         <v>509</v>
@@ -5624,22 +5624,22 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>20.4</v>
+        <v>20.39515615041428</v>
       </c>
       <c r="H5" t="n">
-        <v>28</v>
+        <v>28.17080943275972</v>
       </c>
       <c r="I5" t="n">
-        <v>11.79</v>
+        <v>11.78984599513669</v>
       </c>
       <c r="J5" t="n">
-        <v>0.0002</v>
+        <v>0.0002210596124088129</v>
       </c>
       <c r="K5" t="n">
         <v>636.25</v>
       </c>
       <c r="L5" t="n">
-        <v>0.5074</v>
+        <v>0.5074385510996119</v>
       </c>
       <c r="M5" t="n">
         <v>992</v>
@@ -5706,22 +5706,22 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>15.44</v>
+        <v>15.43624161073826</v>
       </c>
       <c r="H6" t="n">
-        <v>31</v>
+        <v>31.3944817300522</v>
       </c>
       <c r="I6" t="n">
-        <v>24.15</v>
+        <v>24.15402567094516</v>
       </c>
       <c r="J6" t="n">
-        <v>0.5866</v>
+        <v>0.5866394399066511</v>
       </c>
       <c r="K6" t="n">
-        <v>9.926600000000001</v>
+        <v>9.926553672316384</v>
       </c>
       <c r="L6" t="n">
-        <v>0.7396</v>
+        <v>0.7396070320579111</v>
       </c>
       <c r="M6" t="n">
         <v>3106</v>
@@ -5776,7 +5776,7 @@
         <v>19.82</v>
       </c>
       <c r="H7" t="n">
-        <v>28</v>
+        <v>28.32</v>
       </c>
       <c r="I7" t="n">
         <v>15.55</v>
@@ -5991,22 +5991,22 @@
         </is>
       </c>
       <c r="G2" s="1" t="n">
-        <v>11.95</v>
+        <v>11.95063332978527</v>
       </c>
       <c r="H2" s="1" t="n">
-        <v>29</v>
+        <v>28.82672926202094</v>
       </c>
       <c r="I2" s="1" t="n">
-        <v>13.27</v>
+        <v>13.27359840706863</v>
       </c>
       <c r="J2" s="1" t="n">
-        <v>1.4755</v>
+        <v>1.475521125007778</v>
       </c>
       <c r="K2" s="1" t="n">
-        <v>4.605</v>
+        <v>4.604991464108609</v>
       </c>
       <c r="L2" s="1" t="n">
-        <v>0.3724</v>
+        <v>0.3724372910920176</v>
       </c>
       <c r="M2" s="1" t="n">
         <v>8644</v>
@@ -6073,22 +6073,22 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>33.97</v>
+        <v>33.97028990249329</v>
       </c>
       <c r="H3" t="n">
-        <v>87</v>
+        <v>86.87476823070044</v>
       </c>
       <c r="I3" t="n">
-        <v>17.87</v>
+        <v>17.87001124549607</v>
       </c>
       <c r="J3" t="n">
-        <v>1.4173</v>
+        <v>1.417345603929039</v>
       </c>
       <c r="K3" t="n">
-        <v>4.603</v>
+        <v>4.60298643565485</v>
       </c>
       <c r="L3" t="n">
-        <v>0.1828</v>
+        <v>0.1827659481160472</v>
       </c>
       <c r="M3" t="n">
         <v>24176</v>
@@ -6156,22 +6156,22 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>6.97</v>
+        <v>6.965125551270159</v>
       </c>
       <c r="H4" t="n">
-        <v>17</v>
+        <v>17.46977168058065</v>
       </c>
       <c r="I4" t="n">
-        <v>13.23</v>
+        <v>13.22784027691927</v>
       </c>
       <c r="J4" t="n">
-        <v>1.6593</v>
+        <v>1.659321300531586</v>
       </c>
       <c r="K4" t="n">
-        <v>3.0544</v>
+        <v>3.054392402331103</v>
       </c>
       <c r="L4" t="n">
-        <v>0.4419</v>
+        <v>0.4419074604110633</v>
       </c>
       <c r="M4" t="n">
         <v>3569</v>
@@ -6238,22 +6238,22 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>41.37</v>
+        <v>41.36759945184802</v>
       </c>
       <c r="H5" t="n">
-        <v>36</v>
+        <v>36.20186292228556</v>
       </c>
       <c r="I5" t="n">
-        <v>48.28</v>
+        <v>48.27674122146251</v>
       </c>
       <c r="J5" t="n">
-        <v>0.8023</v>
+        <v>0.8023177656738903</v>
       </c>
       <c r="K5" t="n">
-        <v>8.2972</v>
+        <v>8.297225501770956</v>
       </c>
       <c r="L5" t="n">
-        <v>0.5472</v>
+        <v>0.5472399439185297</v>
       </c>
       <c r="M5" t="n">
         <v>17651</v>
@@ -6321,22 +6321,22 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>41.82</v>
+        <v>41.81893687707641</v>
       </c>
       <c r="H6" t="n">
-        <v>50</v>
+        <v>49.90656146179402</v>
       </c>
       <c r="I6" t="n">
-        <v>10.41</v>
+        <v>10.40773086662188</v>
       </c>
       <c r="J6" t="n">
-        <v>0.8413</v>
+        <v>0.8413260296625498</v>
       </c>
       <c r="K6" t="n">
-        <v>11.2434</v>
+        <v>11.24342105263158</v>
       </c>
       <c r="L6" t="n">
-        <v>0.1032</v>
+        <v>0.1032401899310803</v>
       </c>
       <c r="M6" t="n">
         <v>970</v>
@@ -6403,22 +6403,22 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>15.02</v>
+        <v>15.01828312728539</v>
       </c>
       <c r="H7" t="n">
-        <v>47</v>
+        <v>46.85704335713042</v>
       </c>
       <c r="I7" t="n">
-        <v>8.279999999999999</v>
+        <v>8.280529953917052</v>
       </c>
       <c r="J7" t="n">
-        <v>1.5156</v>
+        <v>1.515600998463902</v>
       </c>
       <c r="K7" t="n">
-        <v>2.8514</v>
+        <v>2.851436921578178</v>
       </c>
       <c r="L7" t="n">
-        <v>0.1988</v>
+        <v>0.1988332438935725</v>
       </c>
       <c r="M7" t="n">
         <v>-1963</v>
@@ -6485,22 +6485,22 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>13.67</v>
+        <v>13.66594360086768</v>
       </c>
       <c r="H8" t="n">
-        <v>79</v>
+        <v>79.3709327548807</v>
       </c>
       <c r="I8" t="n">
-        <v>12.81</v>
+        <v>12.81269066503966</v>
       </c>
       <c r="J8" t="n">
-        <v>6.5953</v>
+        <v>6.595281675818589</v>
       </c>
       <c r="K8" t="n">
-        <v>1.7139</v>
+        <v>1.713943268078306</v>
       </c>
       <c r="L8" t="n">
-        <v>0.1047</v>
+        <v>0.1046704357105556</v>
       </c>
       <c r="M8" t="n">
         <v>-13347</v>
@@ -6555,7 +6555,7 @@
         <v>15.02</v>
       </c>
       <c r="H9" t="n">
-        <v>47</v>
+        <v>46.86</v>
       </c>
       <c r="I9" t="n">
         <v>13.23</v>
@@ -6770,22 +6770,22 @@
         </is>
       </c>
       <c r="G2" s="1" t="n">
-        <v>23.07</v>
+        <v>23.07288232992184</v>
       </c>
       <c r="H2" s="1" t="n">
-        <v>-44685</v>
+        <v>61.41252040373843</v>
       </c>
       <c r="I2" s="1" t="n">
-        <v>14.34</v>
+        <v>14.33974005030719</v>
       </c>
       <c r="J2" s="1" t="n">
-        <v>6.8088</v>
+        <v>6.808786667718385</v>
       </c>
       <c r="K2" s="1" t="n">
-        <v>1.4008</v>
+        <v>1.400768822479211</v>
       </c>
       <c r="L2" s="1" t="n">
-        <v>0.0704</v>
+        <v>0.07038097917866981</v>
       </c>
       <c r="M2" s="1" t="n">
         <v>35669</v>
@@ -6852,22 +6852,22 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>28.89</v>
+        <v>28.8880112339828</v>
       </c>
       <c r="H3" t="n">
-        <v>-14152</v>
+        <v>62.41380175029464</v>
       </c>
       <c r="I3" t="n">
-        <v>17.99</v>
+        <v>17.99027109750765</v>
       </c>
       <c r="J3" t="n">
-        <v>6.4456</v>
+        <v>6.445624336310825</v>
       </c>
       <c r="K3" t="n">
-        <v>1.3009</v>
+        <v>1.300946133138182</v>
       </c>
       <c r="L3" t="n">
-        <v>0.0675</v>
+        <v>0.06747535915921023</v>
       </c>
       <c r="M3" t="n">
         <v>12547</v>
@@ -6934,22 +6934,22 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>22.73</v>
+        <v>22.73130411725443</v>
       </c>
       <c r="H4" t="n">
-        <v>11952</v>
+        <v>34.69264599658038</v>
       </c>
       <c r="I4" t="n">
-        <v>15.83</v>
+        <v>15.83271240518905</v>
       </c>
       <c r="J4" t="n">
-        <v>8.2491</v>
+        <v>8.249122739980766</v>
       </c>
       <c r="K4" t="n">
-        <v>1.6912</v>
+        <v>1.691203992514036</v>
       </c>
       <c r="L4" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.0720367478374617</v>
       </c>
       <c r="M4" t="n">
         <v>-14556</v>
@@ -7017,22 +7017,22 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>32.39</v>
+        <v>32.38615146611662</v>
       </c>
       <c r="H5" t="n">
-        <v>-13382</v>
+        <v>83.66733645109092</v>
       </c>
       <c r="I5" t="n">
-        <v>14.01</v>
+        <v>14.01301818853291</v>
       </c>
       <c r="J5" t="n">
-        <v>4.0037</v>
+        <v>4.003739266919029</v>
       </c>
       <c r="K5" t="n">
-        <v>1.2364</v>
+        <v>1.236375108447038</v>
       </c>
       <c r="L5" t="n">
-        <v>0.0733</v>
+        <v>0.07325702420450533</v>
       </c>
       <c r="M5" t="n">
         <v>6766</v>
@@ -7099,22 +7099,22 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>19.56</v>
+        <v>19.56369677362945</v>
       </c>
       <c r="H6" t="n">
-        <v>2978</v>
+        <v>38.55469091544986</v>
       </c>
       <c r="I6" t="n">
-        <v>14.25</v>
+        <v>14.25227319776422</v>
       </c>
       <c r="J6" t="n">
-        <v>6.8857</v>
+        <v>6.885742949503957</v>
       </c>
       <c r="K6" t="n">
-        <v>1.8795</v>
+        <v>1.879527055815935</v>
       </c>
       <c r="L6" t="n">
-        <v>0.0888</v>
+        <v>0.08884228106460039</v>
       </c>
       <c r="M6" t="n">
         <v>-17468</v>
@@ -7169,7 +7169,7 @@
         <v>23.07</v>
       </c>
       <c r="H7" t="n">
-        <v>-13382</v>
+        <v>61.41</v>
       </c>
       <c r="I7" t="n">
         <v>14.34</v>

</xml_diff>